<commit_message>
Deployed 78d2c36 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/artifacts/Montgomery2020_PM25_Mucociliary_SOMA.xlsx
+++ b/artifacts/Montgomery2020_PM25_Mucociliary_SOMA.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -469,176 +469,256 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Short Name</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Montgomery2020</t>
+          <t>Montgomery et al. (2020) - Genome-Wide Analysis Reveals Mucociliary</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Title</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Genome-Wide Analysis Reveals Mucociliary Remodeling of the Nasal Airway Epithelium Induced by Urban PM2.5</t>
+          <t>Remodeling of the Nasal Airway Epithelium Induced by Urban PM2.5</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Authors</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Montgomery MT, Sajuthi SP, Cho SH, Everman JL, Rios CL, Goldfarbmuren KC, Jackson ND, Saef B, Cromie M, Eng C, Medina V, Elhawary JR, Oh SS, Rodriguez-Santana J, Vladar EK, Burchard EG, Seibold MA</t>
+          <t>Am J Respir Cell Mol Biol. 2020;63(2):172-184</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Journal</t>
+          <t>DOI</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Am J Respir Cell Mol Biol 2020;63(2):172-184</t>
+          <t>10.1165/rcmb.2019-0454OC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>DOI</t>
+          <t>PMCID</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>10.1165/rcmb.2019-0454OC</t>
+          <t>PMC7397762</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>PMCID</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>PMC7397762</t>
-        </is>
-      </c>
+          <t>Study Design</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>- In vitro</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Primary human nasal airway epithelial cells (AECs) at ALI</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>In Vitro Model</t>
+          <t>- Donors</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Primary human nasal AECs at ALI, 28-32 days differentiation</t>
+          <t>GALA II childhood asthma study (healthy + asthmatic)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>PM2.5 Source</t>
+          <t>- Exposure</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>3 California cities (Bakersfield/Fresno, Sacramento, Yuba City), 2011</t>
+          <t>PM2.5 organic extract (OE) from California urban sites</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>PM2.5 Extract</t>
+          <t>- Doses</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Water-soluble (WE) and organic-soluble (OE) fractions</t>
+          <t>Low (0.045 ug/cm2), Moderate (0.45 ug/cm2), High (4.5 ug/cm2)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Key Concentrations</t>
+          <t>- Acute protocol</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>OE: 0.045, 0.45, 4.5 ug/cm2; WE: 3, 30 ug/cm2</t>
+          <t>2 stimulations 24h apart, harvest 24h after second</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Acute Protocol</t>
+          <t>- Chronic protocol</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>2 stimulations 24h apart, harvest 24h after second</t>
+          <t>5 stimulations over 5 days</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Chronic Protocol</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>5 stimulations over 5 days (high OE dose)</t>
-        </is>
-      </c>
+          <t>Key findings from paper</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Toxicity</t>
+          <t>- Moderate OE</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>&lt;1% by LDH assay at all concentrations</t>
+          <t>424 DEGs (281 up, 143 down), CYP1A1 LFC=6.21</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr"/>
-      <c r="B16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>AhR signaling activation, IL-1 inflammatory program</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>SOMA Assay Types</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>GeneExpressionAssay, GobletCellAssay, FoxJExpressionAssay</t>
+          <t>MUC5AC upregulation (LFC=0.90), mucus secretory cell enrichment</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>- High OE</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>1296 DEGs, ciliary gene downregulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>- Chronic OE</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>MUC5AC+ cells FC=2.88, FOXJ1+ nuclei 75% decrease</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>SPDEF protein 1.5-fold increase, mucin secretion remodeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>PROTOCOLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>GENE EXPRESSION ASSAYS - Acute Stimulation (RNA-seq validated)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>GOBLET CELL ASSAYS - Chronic Stimulation Results</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>FOXJ1 EXPRESSION ASSAYS - Chronic Stimulation</t>
         </is>
       </c>
     </row>
@@ -722,7 +802,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>FOXJ1 downregulation after chronic 5-day PM2.5 OE. mRNA LFC=-0.36 (p=1.92e-2). FOXJ1+ nuclei decreased 75% (p=1.20e-2). Weaker acetylated alpha-tubulin.</t>
+          <t>FOXJ1 downregulation after chronic 5-day PM2.5 OE. mRNA LFC=-0.36 (p=1.92e-2). FOXJ1+ nuclei decreased 75% vs mock (p=1.20e-2). n=3 donors. Weaker acetylated alpha-tubulin staining observed.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -764,7 +844,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>High OE: ciliary assembly module downregulated (p=4.20e-4). FOXJ1, MCIDAS, MYB, TP73, RFX2, RFX3 all decreased. Ciliated cell enrichment Padj=3.57e-118.</t>
+          <t>At high OE dose (4.5 ug/cm2), ciliary assembly module mean expression downregulated (p=4.20e-4). Ciliogenesis TFs FOXJ1, MCIDAS, MYB, TP73, RFX2, RFX3 all decreased. Ciliated cell marker enrichment Padj=3.57e-118.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -812,7 +892,7 @@
     <col width="29" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="27" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
     <col width="36" customWidth="1" min="6" max="6"/>
     <col width="35" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
@@ -879,7 +959,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -889,7 +969,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000187</t>
+          <t>percent (UO:0000187)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -917,7 +997,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -946,7 +1026,7 @@
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
@@ -995,11 +1075,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>MolecularAssayProtocol</t>
-        </is>
-      </c>
+      <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -1019,11 +1095,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>MolecularAssayProtocol</t>
-        </is>
-      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -1043,11 +1115,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>MolecularAssayProtocol</t>
-        </is>
-      </c>
+      <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -1067,15 +1135,11 @@
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>StainingProtocol</t>
-        </is>
-      </c>
+      <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Confocal microscope; Anti-MUC5AC; Anti-MUC5B; Anti-FOXJ1; Anti-acetylated alpha-tubulin; DAPI</t>
+          <t>Confocal microscope; Anti-MUC5AC antibody; Anti-MUC5B antibody; Anti-FOXJ1 antibody; Anti-acetylated alpha-tubulin antibody; DAPI</t>
         </is>
       </c>
     </row>
@@ -1091,11 +1155,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>MolecularAssayProtocol</t>
-        </is>
-      </c>
+      <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -1115,11 +1175,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>StainingProtocol</t>
-        </is>
-      </c>
+      <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -1147,7 +1203,7 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="27" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="23" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
@@ -1222,7 +1278,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000274</t>
+          <t>microgram per square centimeter (UO:0000274)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -1232,19 +1288,19 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000032</t>
+          <t>hour (UO:0000032)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>EXPOSURE:montgomery-high-oe</t>
+          <t>EXPOSURE:montgomery-chronic-oe</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>PM2.5 organic extract 4.5 ug/cm2 (high dose)</t>
+          <t>PM2.5 organic extract chronic 5-day stimulation (high OE dose)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1264,29 +1320,29 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000274</t>
+          <t>microgram per square centimeter (UO:0000274)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000032</t>
+          <t>hour (UO:0000032)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>EXPOSURE:montgomery-chronic-oe</t>
+          <t>EXPOSURE:montgomery-high-oe</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>PM2.5 organic extract chronic 5-day stimulation (high OE dose)</t>
+          <t>PM2.5 organic extract 4.5 ug/cm2 (high dose)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1306,17 +1362,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000274</t>
+          <t>microgram per square centimeter (UO:0000274)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>120</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000032</t>
+          <t>hour (UO:0000032)</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1393,7 @@
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
   </cols>
@@ -1380,11 +1436,7 @@
           <t>AhR pathway activation</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>CYP1A1 induction by PAH components of PM2.5</t>
-        </is>
-      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>activated</t>
@@ -1407,11 +1459,7 @@
           <t>IL-1 inflammatory program activation</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>IL1A/IL1B hub cytokine network driving epithelial inflammation</t>
-        </is>
-      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>increased</t>
@@ -1434,11 +1482,7 @@
           <t>Goblet cell hyperplasia</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>MUC5AC upregulation, mucus secretory cell enrichment</t>
-        </is>
-      </c>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>increased</t>
@@ -1461,11 +1505,7 @@
           <t>Club cell marker loss</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>SCGB1A1 downregulation indicating loss of club cell identity</t>
-        </is>
-      </c>
+      <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>decreased</t>
@@ -1488,11 +1528,7 @@
           <t>Altered ciliogenesis</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>FOXJ1 downregulation and loss of ciliated cells</t>
-        </is>
-      </c>
+      <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>decreased</t>
@@ -1521,7 +1557,7 @@
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
@@ -1630,11 +1666,7 @@
           <t>Primary nasal AEC ALI culture - GALA II donors</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Acute stimulation model (12 donors)</t>
-        </is>
-      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>CellularSystem</t>
@@ -1659,7 +1691,7 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>UBERON:0001707</t>
+          <t>nasal cavity (UBERON:0001707)</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -1694,19 +1726,15 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>soma:montgomery-culture-high</t>
+          <t>soma:montgomery-culture-chronic</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Primary nasal AEC ALI culture - high OE dose</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>High dose acute model (5 donors)</t>
-        </is>
-      </c>
+          <t>Primary nasal AEC ALI culture - chronic stimulation</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>CellularSystem</t>
@@ -1714,16 +1742,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>nasal epithelial cell</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>nasal epithelial cell</t>
-        </is>
-      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>CL:0002603</t>
@@ -1731,7 +1755,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>UBERON:0001707</t>
+          <t>nasal cavity (UBERON:0001707)</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -1759,26 +1783,22 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>5 donors from GALA II study</t>
+          <t>4-5 donors from GALA II study</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>soma:montgomery-culture-chronic</t>
+          <t>soma:montgomery-culture-high</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Primary nasal AEC ALI culture - chronic stimulation</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>5-day chronic stimulation model (4-5 donors)</t>
-        </is>
-      </c>
+          <t>Primary nasal AEC ALI culture - high OE dose</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>CellularSystem</t>
@@ -1786,26 +1806,18 @@
       </c>
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>nasal epithelial cell</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>nasal epithelial cell</t>
-        </is>
-      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>CL:0002603</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>UBERON:0001707</t>
-        </is>
-      </c>
+      <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Homo sapiens</t>
@@ -1831,7 +1843,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>4-5 donors from GALA II study</t>
+          <t>5 donors from GALA II study</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1863,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="37" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
@@ -1928,12 +1940,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>CYP1A1 mRNA - moderate OE</t>
+          <t>CYP1A1 mRNA - moderate OE dose</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Most highly upregulated gene; AhR pathway activation by PAH components</t>
+          <t>CYP1A1 induction by PM2.5 organic extract at moderate dose (0.45 ug/cm2). LFC=6.21, the most highly upregulated gene. Marker of AhR pathway activation by PAH components.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1985,12 +1997,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>IL1A mRNA - moderate OE</t>
+          <t>IL1A mRNA - moderate OE dose</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Hub cytokine driving broader epithelial inflammatory response</t>
+          <t>IL1A upregulation by PM2.5 OE at moderate dose. LFC=0.91. Identified as hub cytokine driving broader epithelial inflammatory response.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2042,12 +2054,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>IL1B mRNA - moderate OE</t>
+          <t>IL1B mRNA - moderate OE dose</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hub cytokine; drives mucus metaplasia via SPDEF/FOXA3/XBP1</t>
+          <t>IL1B upregulation by PM2.5 OE at moderate dose. LFC=1.22. Hub cytokine in inflammatory network driving mucus metaplasia.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2094,32 +2106,32 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-muc5ac-mod</t>
+          <t>GE:montgomery-spdef-chronic</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>MUC5AC mRNA - moderate OE (RNA-seq)</t>
+          <t>SPDEF mRNA - chronic OE stimulation</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Mucus secretory cell enrichment Padj=1.19e-74</t>
+          <t>SPDEF upregulation after 5-day chronic PM2.5 OE stimulation. LFC=0.84 (p=3.19e-2). Master transcription factor for mucus metaplasia.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>PR:000011230</t>
+          <t>PR:000014070</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>RNA-seq</t>
+          <t>qRT-PCR</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>DESeq2 median of ratios</t>
+          <t>housekeeping gene</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -2129,17 +2141,17 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>soma:montgomery-culture-001</t>
+          <t>soma:montgomery-culture-chronic</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>EXPOSURE:montgomery-mod-oe</t>
+          <t>EXPOSURE:montgomery-chronic-oe</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>PROTOCOL:montgomery-rnaseq-001</t>
+          <t>PROTOCOL:montgomery-qpcr-001; PROTOCOL:montgomery-wb-001</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -2151,52 +2163,52 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-muc2-mod</t>
+          <t>GE:montgomery-scgb1a1-chronic</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MUC2 mRNA - moderate OE (RNA-seq)</t>
+          <t>SCGB1A1 mRNA - chronic OE stimulation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Mucin gene upregulated at moderate dose</t>
+          <t>SCGB1A1 (club cell marker) downregulation after chronic PM2.5 OE. LFC=-1.51 (p=2.94e-2). Indicates loss of club cell identity.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>PR:000011228</t>
+          <t>PR:000014857</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>RNA-seq</t>
+          <t>qRT-PCR</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>DESeq2 median of ratios</t>
+          <t>housekeeping gene</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>KE:ke2-goblet-hyperplasia</t>
+          <t>KE:ke-club-cell-loss</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>soma:montgomery-culture-001</t>
+          <t>soma:montgomery-culture-chronic</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>EXPOSURE:montgomery-mod-oe</t>
+          <t>EXPOSURE:montgomery-chronic-oe</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>PROTOCOL:montgomery-rnaseq-001</t>
+          <t>PROTOCOL:montgomery-qpcr-001</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -2208,32 +2220,32 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-spdef-chronic</t>
+          <t>GE:montgomery-muc5ac-mod</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SPDEF mRNA - chronic OE stimulation</t>
+          <t>MUC5AC mRNA - moderate OE dose (RNA-seq)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Master TF for mucus metaplasia; protein 1.5-fold by WB</t>
+          <t>MUC5AC upregulation by PM2.5 OE at moderate dose. LFC=0.90. Part of mucus secretory cell enrichment (Padj=1.19e-74).</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>PR:000014070</t>
+          <t>PR:000011230</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>qRT-PCR</t>
+          <t>RNA-seq</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>housekeeping gene</t>
+          <t>DESeq2 median of ratios</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -2243,17 +2255,17 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>soma:montgomery-culture-chronic</t>
+          <t>soma:montgomery-culture-001</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>EXPOSURE:montgomery-chronic-oe</t>
+          <t>EXPOSURE:montgomery-mod-oe</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>PROTOCOL:montgomery-qpcr-001; PROTOCOL:montgomery-wb-001</t>
+          <t>PROTOCOL:montgomery-rnaseq-001</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -2265,52 +2277,52 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-scgb1a1-chronic</t>
+          <t>GE:montgomery-muc2-mod</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SCGB1A1 mRNA - chronic OE stimulation</t>
+          <t>MUC2 mRNA - moderate OE dose (RNA-seq)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Club cell marker loss after chronic PM2.5 OE; LFC=-1.51 (p=2.94e-2)</t>
+          <t>MUC2 upregulation by PM2.5 OE at moderate dose. LFC=1.34.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>PR:000014857</t>
+          <t>PR:000011228</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>qRT-PCR</t>
+          <t>RNA-seq</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>housekeeping gene</t>
+          <t>DESeq2 median of ratios</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>KE:ke-club-cell-loss</t>
+          <t>KE:ke2-goblet-hyperplasia</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>soma:montgomery-culture-chronic</t>
+          <t>soma:montgomery-culture-001</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>EXPOSURE:montgomery-chronic-oe</t>
+          <t>EXPOSURE:montgomery-mod-oe</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>PROTOCOL:montgomery-qpcr-001</t>
+          <t>PROTOCOL:montgomery-rnaseq-001</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -2338,9 +2350,9 @@
     <col width="38" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
     <col width="31" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="29" customWidth="1" min="10" max="10"/>
@@ -2417,7 +2429,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
@@ -2449,7 +2461,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -2481,7 +2493,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -2497,55 +2509,63 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-muc5ac-mod-output</t>
+          <t>GE:montgomery-spdef-chronic-output</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>MUC5AC moderate OE RNA-seq measurement</t>
+          <t>SPDEF chronic OE measurement</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>0.90</t>
+          <t>0.84</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
+          <t>fold change (STATO:0000169)</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>fold change (STATO:0000169)</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-muc5ac-mod</t>
+          <t>GE:montgomery-spdef-chronic</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-muc2-mod-output</t>
+          <t>GE:montgomery-scgb1a1-chronic-output</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MUC2 moderate OE RNA-seq measurement</t>
+          <t>SCGB1A1 chronic OE measurement</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>-1.51</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
@@ -2554,70 +2574,62 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-muc2-mod</t>
+          <t>GE:montgomery-scgb1a1-chronic</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-spdef-chronic-output</t>
+          <t>GE:montgomery-muc5ac-mod-output</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>SPDEF chronic OE measurement</t>
+          <t>MUC5AC moderate OE RNA-seq measurement</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.90</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>UO:0000193</t>
-        </is>
-      </c>
+          <t>fold change (STATO:0000169)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-spdef-chronic</t>
+          <t>GE:montgomery-muc5ac-mod</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-scgb1a1-chronic-output</t>
+          <t>GE:montgomery-muc2-mod-output</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SCGB1A1 chronic OE measurement</t>
+          <t>MUC2 moderate OE RNA-seq measurement</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>-1.51</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
@@ -2626,7 +2638,7 @@
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>GE:montgomery-scgb1a1-chronic</t>
+          <t>GE:montgomery-muc2-mod</t>
         </is>
       </c>
     </row>
@@ -2710,7 +2722,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Chronic 5-day PM2.5 OE. MUC5AC mRNA LFC=1.72 (p=1.27e-2). MUC5AC+ cells FC=2.88 (p=3.19e-2). MUC5AC secretion FC=2.2 (p=1.54e-2).</t>
+          <t>Chronic 5-day PM2.5 OE stimulation. MUC5AC mRNA LFC=1.72 (p=1.27e-2). MUC5AC+ cells FC=2.88 (p=3.19e-2). MUC5AC secretion FC=2.2 (p=1.54e-2). All 4 donors showed increase in MUC5AC+ cells.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2752,7 +2764,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Chronic 5-day PM2.5 OE. MUC5B mRNA LFC=-0.72 (p=9.74e-2, trend). MUC5B+ cells FC=0.74 (p=8.84e-2). MUC5B secretion FC=0.81 (p=3.59e-3).</t>
+          <t>Chronic 5-day PM2.5 OE stimulation. MUC5B mRNA LFC=-0.72 (p=9.74e-2, trend). MUC5B+ cells FC=0.74 (p=8.84e-2). MUC5B secretion FC=0.81 (p=3.59e-3). All 4 donors showed MUC5B+ cell decrease.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2794,7 +2806,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>AB-PAS staining. Average FC=2.01 in mucin-positive cells (p=6.52e-2). 3 of 4 donors showed increase.</t>
+          <t>AB-PAS staining after chronic 5-day PM2.5 OE stimulation. Average FC=2.01 in mucin-positive cells (p=6.52e-2). 3 of 4 donors showed increase.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2836,7 +2848,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>MUC5AC/MUC5B ratio significantly increased at moderate OE dose (p=3.19e-2). MUC5AC LFC=0.90 with MUC5B trending down.</t>
+          <t>MUC5AC/MUC5B ratio significantly increased at moderate OE dose (p=3.19e-2). MUC5AC LFC=0.90 with MUC5B trending down (LFC=-0.79 at high dose, Padj=1.0e-1).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2886,15 +2898,15 @@
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
     <col width="31" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="27" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
     <col width="30" customWidth="1" min="12" max="12"/>
     <col width="29" customWidth="1" min="13" max="13"/>
     <col width="26" customWidth="1" min="14" max="14"/>
-    <col width="25" customWidth="1" min="15" max="15"/>
+    <col width="27" customWidth="1" min="15" max="15"/>
     <col width="29" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
@@ -3001,7 +3013,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -3011,7 +3023,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -3025,7 +3037,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -3059,7 +3071,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -3069,7 +3081,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
@@ -3099,7 +3111,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -3139,7 +3151,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -3151,7 +3163,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>UO:0000193</t>
+          <t>fold change (STATO:0000169)</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr"/>

</xml_diff>